<commit_message>
chore(sites): gen-site 二轮配通 raybiotech/cas9x，台账补站点链接
</commit_message>
<xml_diff>
--- a/data/seeds/gen-site-template.xlsx
+++ b/data/seeds/gen-site-template.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -529,27 +529,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>acrobiosystems.com</t>
+          <t>promega.com.cn</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.acrobiosystems.com/category/kits-assay-reagents/elisa-kit</t>
+          <t>https://www.promega.com.cn/products/cell-health-assays/inflammation-assay/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>北京百普赛斯生物科技股份有限公司</t>
+          <t>普洛麦格(北京)生物技术有限公司</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACROBiosystems 百普赛斯</t>
+          <t>Promega</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -561,22 +561,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>abcam.com</t>
+          <t>rndsystems.com</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.abcam.com/en-us/products/primary-antibodies</t>
+          <t>https://www.rndsystems.com/products/elisas/quantikine-colorimetric-sandwich-elisa</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Abcam plc</t>
+          <t>Bio-Techne Corporation (R&amp;D Systems)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Abcam</t>
+          <t>R&amp;D Systems</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -593,22 +593,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bdbiosciences.com</t>
+          <t>raybiotech.com</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.bdbiosciences.com/en-sg/products/reagents/flow-cytometry-reagents/research-reagents</t>
+          <t>https://www.raybiotech.com/elisa-kits-products/sandwich-elisa</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Becton, Dickinson and Company (BD Biosciences)</t>
+          <t>RayBiotech, Inc.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BD Biosciences</t>
+          <t>RayBiotech</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -625,27 +625,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>beckman.com</t>
+          <t>cas9x.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.beckman.com/reagents/coulter-flow-cytometry/antibodies-and-kits</t>
+          <t>https://www.cas9x.com/bdxb</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Beckman Coulter, Inc.</t>
+          <t>苏州海星生物科技有限公司</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Beckman Coulter</t>
+          <t>cas9x 海星生物</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -657,22 +657,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cellsignal.com</t>
+          <t>acrobiosystems.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.cellsignal.com/browse?tab=product&amp;categories=Primary%20Antibodies</t>
+          <t>https://www.acrobiosystems.com/category/kits-assay-reagents/elisa-kit</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Cell Signaling Technology, Inc.</t>
+          <t>北京百普赛斯生物科技股份有限公司</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CST</t>
+          <t>ACROBiosystems 百普赛斯</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -681,518 +681,6 @@
         </is>
       </c>
       <c r="I6" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>caymanchem.com</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.caymanchem.com/assays</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Cayman Chemical Company</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Cayman Chemical</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>miltenyibiotec.com</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.miltenyibiotec.com/US-en/products/macs-cell-separation.html</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Miltenyi Biotec GmbH</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Miltenyi</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>promega.com.cn</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.promega.com.cn/products/cell-health-assays/</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>普洛麦格(北京)生物技术有限公司</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Promega</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>rndsystems.com</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.rndsystems.com/products/elisas</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Bio-Techne Corporation (R&amp;D Systems)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>R&amp;D Systems</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>raybiotech.com</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://www.raybiotech.com/elisa-kits</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>RayBiotech, Inc.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>RayBiotech</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>sciencellonline.com</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://sciencellonline.com/en/products-services/cell-culture-media/</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ScienCell Research Laboratories, Inc.</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>ScienCell</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>selleckchem.com</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://www.selleckchem.com/screening-libraries.html</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Selleck Chemicals LLC</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Selleck</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>basalmedia.com</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://www.basalmedia.com/</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>上海源培生物科技股份有限公司</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>BasalMedia 源培生物</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>senbeijia.com</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>http://www.senbeijia.com/category.php?id=58</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>南京森贝伽生物科技有限公司</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Senbeijia 森贝伽</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>dojindo.cn</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://www.dojindo.cn/#/index</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>同仁化学研究所 (Dojindo Laboratories)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Dojindo 同仁化学</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>corning.com</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://www.corning.com/cn/zh/products/life-sciences/products/cell-Culture.html</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Corning Incorporated (Corning Life Sciences)</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Corning</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>lonsera.cn</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>https://www.lonsera.cn/list_11/</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>苏州双洳生物科技有限公司</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Lonsera 双洳生物</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>cas9x.com</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://www.cas9x.com/bdxb</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>苏州海星生物科技有限公司</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>cas9x 海星生物</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>thermofisher.com</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://www.thermofisher.com/mx/en/home/life-science/antibodies/ebioscience.html</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Thermo Fisher Scientific Inc.</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Thermo Fisher</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>novoprotein.com.cn</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://www.novoprotein.com.cn/products</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>苏州近岸蛋白质科技股份有限公司</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Novoprotein 近岸蛋白</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>genscript.com</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>https://www.genscript.com/catalog-antibody-products.html</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>南京金斯瑞生物科技有限公司</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>GenScript 金斯瑞</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
         <is>
           <t>browser</t>
         </is>
@@ -1410,7 +898,6 @@
           <t>使用步骤</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>1) 在「站点清单」按列填入真实站点（删除示例行）</t>
@@ -1418,8 +905,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>2) 运行 pnpm gen-site:batch  （默认读取 data/seeds/gen-site-template.xlsx）</t>
@@ -1427,8 +912,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>3) 可用 pnpm gen-site:batch --file &lt;路径&gt; 指定其它 Excel</t>
@@ -1436,8 +919,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>4) 加 --dry-run 仅解析并打印待生成清单，不调用模型</t>
@@ -1445,22 +926,18 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>5) 每个站点生成后产出 config/sites/&lt;domain&gt;.yaml，再 pnpm probe 验证</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>config/sites/ 目录是爬取范围的唯一真相源（crawl 默认 --source config）：</t>
@@ -1468,8 +945,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>放一个 &lt;domain&gt;.yaml 就爬一个站，删掉就不爬；本 Excel 只是把站点信息喂给模型生成 YAML 的辅助工具。</t>

</xml_diff>